<commit_message>
Update published master datasets (2026-02-26)
</commit_message>
<xml_diff>
--- a/archive/InnovateUK_Funding_Opportunities_WeeklyBreakdown_2026-02-26.xlsx
+++ b/archive/InnovateUK_Funding_Opportunities_WeeklyBreakdown_2026-02-26.xlsx
@@ -482,13 +482,13 @@
         <v>46078</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -8010,7 +8010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8323,6 +8323,295 @@
         <v>46078</v>
       </c>
       <c r="O5" s="1" t="n">
+        <v>46078</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ARIA: Universal Fabricators - concept papers</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/aria-universal-fabricators-concept-papers/</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-02-26 10:34</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>46079.44027777778</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>16/02/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>46069</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>09/03/2026                              14:00</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>46090.58333333334</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>£50</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="O6" s="1" t="n">
+        <v>46078</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ADOPT Facilitator Support Grant: Round 7</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/adopt-facilitator-support-grant-round-7/</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-02-26 10:34</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>46079.44027777778</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>26/02/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>46079</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>08/04/2026                              11:00</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>46120.45833333334</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>£100,000</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="O7" s="1" t="n">
+        <v>46078</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>UK Defence Innovation Competition: Innovation Support to Operations Phase 3 (Cycle 7)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/uk-defence-innovation-competition-innovation-support-to-operations-phase-3-cycle-7/</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-02-26 10:34</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>46079.44027777778</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>23/02/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>46076</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>12/05/2026                              12:00</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>46154.5</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>£1.0 million</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="O8" s="1" t="n">
+        <v>46078</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Countering Illegal Use of UAS Around Prisons and Sensitive Sites</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/countering-illegal-use-of-uas-around-prisons-and-sensitive-sites/</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-02-26 10:34</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>46079.44027777778</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>16/02/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>46069</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>31/03/2026                              12:00</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>46112.5</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>£5,000</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="O9" s="1" t="n">
+        <v>46078</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ADOPT Facilitator Support Grant: Round 7</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2404/overview/99693fa4-0f17-4de8-b812-34f2be37a4d0</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-02-26 10:40</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>46079.44444444445</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Wednesday 8 April 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>46120.45833333334</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>£2,500</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="O10" s="1" t="n">
         <v>46078</v>
       </c>
     </row>

</xml_diff>